<commit_message>
sedo: draft1 refreshed to 1,320 after Dynadot completeness closed at 453 (+overhead-cranes.com, +paper-cups.com; diff is exactly the 2 rows)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agent_docs/docs024_key_docs_latest/sedo_domain_management/outbound/SEDO_IMPORT_2026-09-02_draft1.xlsx
+++ b/docs/agent_docs/docs024_key_docs_latest/sedo_domain_management/outbound/SEDO_IMPORT_2026-09-02_draft1.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="1327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1329" uniqueCount="1329">
   <si>
     <t>Domain Name</t>
   </si>
@@ -2491,6 +2491,9 @@
     <t>overclad.com</t>
   </si>
   <si>
+    <t>overhead-cranes.com</t>
+  </si>
+  <si>
     <t>overmaken.com</t>
   </si>
   <si>
@@ -2519,6 +2522,9 @@
   </si>
   <si>
     <t>palatschinken.com</t>
+  </si>
+  <si>
+    <t>paper-cups.com</t>
   </si>
   <si>
     <t>parallelled.com</t>
@@ -18542,6 +18548,28 @@
         <v>9</v>
       </c>
     </row>
+    <row r="1320">
+      <c r="A1320" t="s">
+        <v>1327</v>
+      </c>
+      <c r="B1320" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1320" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B1321" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1321" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>